<commit_message>
新增: 環保餐廳 query_charts 補上 newtaipei row (對齊綠色商店 3-city 結構)
原本只有 metrotaipei (跨市 UNION) 與 taipei 兩 row,缺單獨呈現新北的條目。
補一筆 city=newtaipei row,結構鏡像 taipei row:
  - source: 新北市政府環保局
  - short_desc: 新北環保餐廳家數
  - links: data.ntpc dataset e90d14f8-…
  - contributors: {ntpc}
  - query_chart: SELECT '新北市'…FROM eco_friendly_restaurant_ntpe

CSV 與 xlsx 同步更新,xlsx 由 csv 重新打包。
</commit_message>
<xml_diff>
--- a/Taipei-City-Dashboard-DE/component-meta/eco_diet_restaurants_points/eco_diet_restaurants_points.xlsx
+++ b/Taipei-City-Dashboard-DE/component-meta/eco_diet_restaurants_points/eco_diet_restaurants_points.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T3"/>
+  <dimension ref="A1:T4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -716,6 +716,76 @@
       <c r="T3" t="inlineStr">
         <is>
           <t>taipei</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>eco_diet_restaurants_points</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>static</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>新北市政府環保局</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>新北環保餐廳家數</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>新北市政府環保局公告之環保餐廳當前清單統計，以「家」為單位呈現新北市環保飲食店家總量。</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>市民查詢居家附近環保餐廳供給度、店家規劃新分店時參考既有環保認證店家分布。</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>{https://data.ntpc.gov.tw/datasets/e90d14f8-5995-4ebb-af19-8f8fd7d396c8}</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>{ntpc}</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>two_d</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>SELECT '新北市' AS x_axis, COUNT(*)::float AS data FROM eco_friendly_restaurant_ntpe</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>newtaipei</t>
         </is>
       </c>
     </row>

</xml_diff>